<commit_message>
feat: corregir y simplificar exportación de descuentos en Excel y PDF
</commit_message>
<xml_diff>
--- a/backend/data/exports/CM-PROF-TEST-05 - Validación Export Institucional.xlsx
+++ b/backend/data/exports/CM-PROF-TEST-05 - Validación Export Institucional.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>PROYECTO: CM-PROF-TEST-05-Validación Export Institucional</t>
   </si>
@@ -46,7 +46,7 @@
     <t>TIEMPO EJECUCIÓN</t>
   </si>
   <si>
-    <t>12</t>
+    <t>12 días</t>
   </si>
   <si>
     <t>FECHA</t>
@@ -143,9 +143,6 @@
   </si>
   <si>
     <t>mario.lincango@construmetrica.com</t>
-  </si>
-  <si>
-    <t>Validación digital</t>
   </si>
 </sst>
 </file>
@@ -155,7 +152,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -166,63 +163,35 @@
     <font>
       <b/>
       <color rgb="FF444242"/>
-      <sz val="11"/>
-      <name val="Gotham Black"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF444242"/>
-      <sz val="14"/>
+      <sz val="12"/>
       <name val="Gotham Black"/>
     </font>
     <font>
       <color rgb="FF444242"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Gotham Book"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF444242"/>
-      <sz val="9"/>
-      <name val="Gotham Black"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Gotham Black"/>
     </font>
     <font>
       <b/>
       <color rgb="FF550012"/>
-      <sz val="10"/>
+      <sz val="12"/>
       <name val="Gotham Black"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF444242"/>
-      <sz val="10"/>
-      <name val="Gotham Black"/>
-    </font>
-    <font>
-      <color rgb="FF444242"/>
-      <sz val="10"/>
-      <name val="Gotham Book"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFFF0033"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Gotham Black"/>
     </font>
     <font>
       <color rgb="FF777777"/>
-      <sz val="9"/>
-      <name val="Gotham Book"/>
-    </font>
-    <font>
-      <color rgb="FF444242"/>
-      <sz val="8"/>
+      <sz val="12"/>
       <name val="Gotham Book"/>
     </font>
   </fonts>
@@ -271,60 +240,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -349,7 +319,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>28000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>28000</xdr:rowOff>
+      <xdr:rowOff>32000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1238250" cy="400050"/>
     <xdr:pic>
@@ -385,10 +355,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>70000</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6999</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>57600</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="857250" cy="857250"/>
     <xdr:pic>
@@ -750,7 +720,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -761,7 +731,7 @@
     <col min="6" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -770,7 +740,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -803,26 +773,14 @@
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-    </row>
+    <row r="5" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -831,11 +789,11 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -844,11 +802,11 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
@@ -857,100 +815,90 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+    <row r="14" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C15" s="9">
         <v>5</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="11">
-        <v>2</v>
-      </c>
-      <c r="F14" s="12">
-        <v>500</v>
-      </c>
-      <c r="G14" s="12">
-        <f>E14*F14</f>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="9">
-        <v>7</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>25</v>
       </c>
       <c r="E15" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="12">
         <v>500</v>
@@ -959,35 +907,45 @@
         <f>E15*F15</f>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="14">
-        <f>SUM(C14,C15)</f>
+    <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="9">
+        <v>7</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="11">
+        <v>1</v>
+      </c>
+      <c r="F16" s="12">
+        <v>500</v>
+      </c>
+      <c r="G16" s="12">
+        <f>E16*F16</f>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
-      <c r="G18" s="15">
-        <f>SUM(G14,G15)</f>
+      <c r="G18" s="14">
+        <f>SUM(C15,C16)</f>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -995,47 +953,49 @@
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
       <c r="G19" s="15">
+        <f>SUM(G15,G16)</f>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="15">
         <v>225</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17">
-        <f>G18+G19</f>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17">
+        <f>G19+G20</f>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
         <v>32</v>
-      </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-    </row>
-    <row r="24" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>33</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -1044,9 +1004,9 @@
       <c r="F24" s="19"/>
       <c r="G24" s="19"/>
     </row>
-    <row r="25" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="19"/>
       <c r="C25" s="19"/>
@@ -1055,9 +1015,9 @@
       <c r="F25" s="19"/>
       <c r="G25" s="19"/>
     </row>
-    <row r="26" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
@@ -1066,9 +1026,9 @@
       <c r="F26" s="19"/>
       <c r="G26" s="19"/>
     </row>
-    <row r="27" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="19"/>
@@ -1079,7 +1039,7 @@
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -1088,31 +1048,31 @@
       <c r="F28" s="19"/>
       <c r="G28" s="19"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
+    <row r="29" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1123,7 +1083,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -1134,7 +1094,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1145,7 +1105,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -1154,19 +1114,24 @@
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="20" t="s">
-        <v>44</v>
-      </c>
-    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+    </row>
+    <row r="38" ht="15.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="37">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:G5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="A7:B7"/>
@@ -1175,31 +1140,33 @@
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="C9:G9"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A36:G36"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>